<commit_message>
Update database.xlsx sample to match the current sheet schema
The sample workbook was still the very first version from early in the
project (3 sheets, ~13 Members columns, no 事業責任者 role) and no
longer matched gas/README.md's documented column list, which has
grown across many rounds (talent management, task management fields,
project members/owner, role hierarchy, etc).

Rebuilt Members/Projects/Tasks with the exact current column names and
order from the README, refreshed the example rows (including a
事業責任者 example member) and 使い方 sheet text, and added an optional
Settings sheet showing the key/value sync format from README §4.6.

Also fixed two stale passages in gas/README.md's role/scope
description and known-limitations section that still described the
old "only the single top role is full admin" model, superseded by the
事業責任者/代表 parity change.
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="使い方" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Members" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,21 +31,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <name val="Arial"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -79,12 +70,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -464,68 +454,176 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Members: role列は「代表」「班長」「一般」のいずれか。</t>
+          <t>Members: role列は「一般」、またはAdmin → Tagsで自由に追加できる権限レベル</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  project_ids: 班長が担当するプロジェクトID（複数可、カンマ区切り）。代表・一般は空欄でよい。</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  （初期値：班長・事業責任者・代表、この順に上位）。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  「一般」以外はすべて何らかの管理者権限を持ちます。権限レベルのうち最下位</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Projects: プロジェクトの一覧。</t>
+          <t xml:space="preserve">  （初期値では「班長」）以外は組織全体のAdmin画面にフルアクセスでき、最下位の</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ロールだけがAdmin → Membersの「担当プロジェクト」で指定した範囲に限定されます。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Tasks: status/assign_type/visibilityは指定の値のみを使用。</t>
+          <t xml:space="preserve">  project_ids: 最下位の管理者ロール（例：班長）が担当するプロジェクトID</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  （複数可、カンマ区切り）。それ以外のロール・一般は空欄でよい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  *_json列（career_history_json など）はJSON文字列です。空欄のままでも動作します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Projects: プロジェクトの一覧。type列はAdmin → Projectsのテンプレート機能に使われます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Tasks: status/assign_type/visibility/difficulty/priority/importanceは指定の値のみを使用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  status: 未着手 / 進行中 / サポート必要 / 確認待ち / 修正中 / 完了</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  assign_type: open_bid / manager_assign / request / personal</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  visibility: 全員 / 班長以上</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  visibility: 全員 / 幹部（幹部＝一般以外の全権限レベル）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  difficulty: 新人歓迎 / 少し経験必要 / 経験者向け</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  priority: 高 / 中 / 低</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  importance: 一般 / 重要 / 対外公開（空欄は一般扱い。重要・対外公開は最下位以外の</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    管理者ロール（初期値では事業責任者・代表）のみが承認できます）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  approval_status: 承認待ち / 承認済み（空欄は承認済み扱い）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Settings（任意）: key/valueの2列。INPUT画面の選択肢やAdmin → Tagsの設定を</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  スプレッドシート経由で全員の画面に同期したい場合に追加します。詳細は</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gas/README.md の「4.6. 選択肢プールのスプレッドシート同期」を参照してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>列名の詳細な意味は gas/README.md の「1. シートの列構成」を参照してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>黄色い行は入力例です。実データを入れる際は書き換え・削除してください。</t>
         </is>
@@ -542,190 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>project_ids</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>will_tags</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>judgment_tags</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>（例）山田太郎</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>代表</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>宇宙工学,広報</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>リーダーシップ,調整力</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>（例）鈴木花子</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>班長</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>1,3</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>UI/UX,デザイン</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>丁寧,締切厳守</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>（例）佐藤次郎</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>プログラミング</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>（例）Cosmo Base</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>宇宙テーマのメディア・コミュニティサイト開発</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -742,127 +657,940 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>project_ids</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>will_tags</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>judgment_tags</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>notify_new_task</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>reports_to_id</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>mentor_id</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>unavailable_dates</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>avatar_color</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>avatar_initials</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>avatar_url</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>years_of_experience</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>has_management_experience</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>desired_areas</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>career_history_json</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>qualifications_json</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>evaluation_history_json</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>transfer_history_json</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>skill_levels_json</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>competencies_json</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>career_aspiration</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>desired_future_role</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>career_plan</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>training_history_json</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>development_plan_json</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>one_on_ones_json</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>（例）山田太郎</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>代表</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>宇宙工学,広報</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>リーダーシップ,調整力</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>yamada@example.com</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>[{"id":"c-1","startDate":"2019-04-01","affiliation":"Orbit","role":"代表","description":"創業"}]</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>[{"id":"q-1","name":"普通自動車免許","obtainedDate":"2015-03-01"}]</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>組織づくりに関わり続けたい</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>（例）鈴木花子</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>事業責任者</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX,デザイン</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>丁寧,締切厳守</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>suzuki@example.com</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>マネジメント</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>{"UI/UX":4,"デザイン":5}</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>事業責任者</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>（例）佐藤次郎</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>班長</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>プログラミング</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>sato@example.com</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-05,2026-09-06</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>開発,設計</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>（例）高橋美咲</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>プログラミング</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>member_ids</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>owner_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>（例）Cosmo Base</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>宇宙テーマのメディア・コミュニティサイト開発</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>コンテンツ開発</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AK3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="20" customWidth="1" min="37" max="37"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>project_id</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>assign_type</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>assignee_id</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>creator_id</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>accepted_at</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>deliverable_url</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>feedback_comment</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>due_time</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>visibility</t>
         </is>
       </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>completed_date</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>last_activity</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>progress_note</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>original_input_id</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>depends_on_ids</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>blocker_note</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>blocker_since</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>deliverables_json</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>history_json</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>comments_json</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>estimated_hours</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>actual_hours</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>retrospective_json</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>importance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>（例）Tシャツを発注する</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>新歓用Tシャツの発注</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>open_bid</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>全員</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>物品調達</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>新人歓迎</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>（例）宇宙ニュース記事を執筆する</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>月刊コラムの記事執筆</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>manager_assign</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>全員</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>広報</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>ライティング</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>ライティング,リサーチ</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>少し経験必要</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>初稿レビュー待ち</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE3" s="3" t="inlineStr">
+        <is>
+          <t>[{"id":"dl-1","label":"初稿Googleドキュメント","url":"https://docs.google.com/..."}]</t>
+        </is>
+      </c>
+      <c r="AH3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK3" s="3" t="inlineStr">
+        <is>
+          <t>重要</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>skill_options</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>デザイン,Canva,ライティング,リサーチ,SNS,広報,コミュニケーション,イベント運営,メール,UI/UX,実装,企画,要件定義,プロダクト設計,校閲</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>category_options</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>未分類,デザイン,渉外,イベント,広報,ライティング,企画,リサーチ,開発,物品調達</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>role_levels</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>班長,事業責任者,代表</t>
         </is>
       </c>
     </row>

</xml_diff>